<commit_message>
In-Class: republish the updated SK hynix FCFF valuation workbook
Philip re-saved 99_SKhynix_FCFF_Valuation_Korean.xlsx; the third valuation sheet
is now named "3) VAL Gordon Growth Model" (was "Goldens").

Excel still had the source file open, so strip_metadata.ps1 could not clean it in
place - Excel had re-stamped cp:lastModifiedBy on save. Published a copy cleaned at
the zip level instead, which leaves every other part byte-identical. The Dropbox
source still carries the stamp, so it needs a strip pass once Excel releases it,
otherwise the next sync-files.ps1 run will overwrite this clean copy with it.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/inclass/korean/IC_L8_skhynix_fcff.xlsx
+++ b/files/inclass/korean/IC_L8_skhynix_fcff.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hong1p\Dropbox\1_0_teaching\0_2026_Summer\0_Kaist MBA\1_weekly notes\0_Valuation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D720615-4C23-405F-94D9-95951CC1930E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFA1E77-4CA2-45CB-8697-D622F0E2CC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2145" windowWidth="29040" windowHeight="15195" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2145" windowWidth="29040" windowHeight="15195" tabRatio="500" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Consensus" sheetId="5" r:id="rId5"/>
     <sheet name="1) DCF Val_FCFF" sheetId="7" r:id="rId6"/>
     <sheet name="2) VAL with Earnings" sheetId="8" r:id="rId7"/>
-    <sheet name="3) VAL Goldens Growth Model" sheetId="9" r:id="rId8"/>
+    <sheet name="3) VAL Gordon Growth Model" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -8299,14 +8299,14 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11741,34 +11741,34 @@
       <c r="A6" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="48" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="C6" s="48" t="s">
         <v>129</v>
       </c>
-      <c r="D6" s="49" t="s">
+      <c r="D6" s="48" t="s">
         <v>130</v>
       </c>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="F6" s="49" t="s">
+      <c r="F6" s="48" t="s">
         <v>132</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="G6" s="48" t="s">
         <v>133</v>
       </c>
-      <c r="H6" s="49" t="s">
+      <c r="H6" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="I6" s="49" t="s">
+      <c r="I6" s="48" t="s">
         <v>135</v>
       </c>
-      <c r="J6" s="49" t="s">
+      <c r="J6" s="48" t="s">
         <v>136</v>
       </c>
-      <c r="K6" s="49" t="s">
+      <c r="K6" s="48" t="s">
         <v>65</v>
       </c>
     </row>
@@ -12392,28 +12392,28 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="51" t="s">
         <v>260</v>
       </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="51"/>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="51" t="s">
         <v>175</v>
       </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
     </row>
     <row r="16" spans="1:4" ht="30" customHeight="1">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="51" t="s">
         <v>176</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
+      <c r="B16" s="51"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -12686,7 +12686,7 @@
       <c r="A27" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="C27" s="49" t="s">
+      <c r="C27" s="48" t="s">
         <v>203</v>
       </c>
       <c r="D27" s="14" t="s">
@@ -12704,7 +12704,7 @@
       <c r="H27" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="I27" s="49" t="s">
+      <c r="I27" s="48" t="s">
         <v>209</v>
       </c>
     </row>
@@ -12728,7 +12728,7 @@
       <c r="H28" s="23">
         <v>0.05</v>
       </c>
-      <c r="L28" s="50" t="s">
+      <c r="L28" s="49" t="s">
         <v>261</v>
       </c>
     </row>
@@ -13513,7 +13513,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="50" t="s">
         <v>265</v>
       </c>
     </row>
@@ -13679,7 +13679,7 @@
       <c r="A27" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="C27" s="49" t="s">
+      <c r="C27" s="48" t="s">
         <v>203</v>
       </c>
       <c r="D27" s="14" t="s">
@@ -13697,7 +13697,7 @@
       <c r="H27" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="I27" s="49" t="s">
+      <c r="I27" s="48" t="s">
         <v>209</v>
       </c>
     </row>
@@ -13780,27 +13780,27 @@
         <v>210</v>
       </c>
       <c r="C31" s="17">
-        <f>C29*C30</f>
+        <f t="shared" ref="C31:H31" si="0">C29*C30</f>
         <v>47206</v>
       </c>
       <c r="D31" s="17">
-        <f>D29*D30</f>
+        <f t="shared" si="0"/>
         <v>199345.644</v>
       </c>
       <c r="E31" s="17">
-        <f>E29*E30</f>
+        <f t="shared" si="0"/>
         <v>197407.56134999997</v>
       </c>
       <c r="F31" s="17">
-        <f>F29*F30</f>
+        <f t="shared" si="0"/>
         <v>83579.814281249986</v>
       </c>
       <c r="G31" s="17">
-        <f>G29*G30</f>
+        <f t="shared" si="0"/>
         <v>87758.804995312501</v>
       </c>
       <c r="H31" s="17">
-        <f>H29*H30</f>
+        <f t="shared" si="0"/>
         <v>89513.981095218769</v>
       </c>
     </row>
@@ -13827,27 +13827,27 @@
         <v>263</v>
       </c>
       <c r="C40" s="38">
-        <f>C31</f>
+        <f t="shared" ref="C40:H40" si="1">C31</f>
         <v>47206</v>
       </c>
       <c r="D40" s="38">
-        <f>D31</f>
+        <f t="shared" si="1"/>
         <v>199345.644</v>
       </c>
       <c r="E40" s="38">
-        <f>E31</f>
+        <f t="shared" si="1"/>
         <v>197407.56134999997</v>
       </c>
       <c r="F40" s="38">
-        <f>F31</f>
+        <f t="shared" si="1"/>
         <v>83579.814281249986</v>
       </c>
       <c r="G40" s="38">
-        <f>G31</f>
+        <f t="shared" si="1"/>
         <v>87758.804995312501</v>
       </c>
       <c r="H40" s="38">
-        <f>H31</f>
+        <f t="shared" si="1"/>
         <v>89513.981095218769</v>
       </c>
     </row>
@@ -14069,7 +14069,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="50" t="s">
         <v>266</v>
       </c>
     </row>
@@ -14235,7 +14235,7 @@
       <c r="A27" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="C27" s="49" t="s">
+      <c r="C27" s="48" t="s">
         <v>203</v>
       </c>
       <c r="D27" s="14" t="s">
@@ -14253,7 +14253,7 @@
       <c r="H27" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="I27" s="49" t="s">
+      <c r="I27" s="48" t="s">
         <v>209</v>
       </c>
     </row>
@@ -14335,27 +14335,27 @@
         <v>263</v>
       </c>
       <c r="C40" s="38">
-        <f>C31</f>
+        <f t="shared" ref="C40:H40" si="0">C31</f>
         <v>0</v>
       </c>
       <c r="D40" s="38">
-        <f>D31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E40" s="38">
-        <f>E31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F40" s="38">
-        <f>F31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G40" s="38">
-        <f>G31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H40" s="38">
-        <f>H31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>